<commit_message>
Fix row spacing in Excel file
https://claude.ai/code/session_01XBmmQd3mYizXfGYhbNjnwy
</commit_message>
<xml_diff>
--- a/leads_ohne_website.xlsx
+++ b/leads_ohne_website.xlsx
@@ -70,35 +70,29 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="00DDDDDD"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -469,16 +463,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
@@ -520,7 +514,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
@@ -534,9 +528,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Ulrich-von-Hutten-Straße 7, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ulrich-von-Hutten-Straße 7, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -554,53 +548,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="5" t="n">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>ELGAWA GmbH Elektro-, Gas- und Wasserinstallationen</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Horststraße 110, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Horststraße 110, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>+49 6341 50589</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
@@ -614,9 +608,9 @@
           <t>Karlsruhe</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Talstraße 8, 76228 Karlsruhe, Deutschland</t>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Talstraße 8, 76228 Karlsruhe</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -634,53 +628,53 @@
           <t>4.6 ★</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="n">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Klaus Plappert Elektroinstallateurmeister</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Karlsruhe</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Beunstraße 59, 76229 Karlsruhe, Deutschland</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Beunstraße 59, 76229 Karlsruhe</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>+49 172 9372422</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Elektroinstallationsdienst</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H5" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
@@ -694,9 +688,9 @@
           <t>Königsbach-Stein</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Rhönstraße 54, 75203 Königsbach-Stein, Deutschland</t>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Rhönstraße 54, 75203 Königsbach-Stein</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -714,53 +708,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="n">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Elektro-Hettich GmbH</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Kuppenheim</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Ringstraße 2, 76456 Kuppenheim, Deutschland</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Ringstraße 2, 76456 Kuppenheim</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>+49 7222 94510</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>Elektriker</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
@@ -774,9 +768,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Arbotstraße 9, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Arbotstraße 9, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -794,53 +788,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="n">
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Matz &amp; Jung GmbH - Gebäudetechnik</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Speyerer Str. 2, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Speyerer Str. 2, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
         <is>
           <t>+49 6341 98570</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>Heizungs- und Klimatechnikbetrieb</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>4.3 ★</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -854,9 +848,9 @@
           <t>Landau an der Isar</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Gewerbegebiet Landauer Wiesen, Siemensstraße 17, 94405 Landau an der Isar, Deutschland</t>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Landauer Wiesen, Siemensstraße 17, 94405 Landau an der Isar</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -874,53 +868,53 @@
           <t>4.1 ★</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="n">
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>F. Letzelter Heizung / Solar / Sanitär</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Kraftgasse 54, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Kraftgasse 54, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>+49 6341 890138</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>Heizungsmonteur</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H11" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -934,9 +928,9 @@
           <t>Stuttgart</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
-        <is>
-          <t>Alexanderstraße 175, 70180 Stuttgart, Deutschland</t>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Alexanderstraße 175, 70180 Stuttgart</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -954,53 +948,53 @@
           <t>4.6 ★</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="n">
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>Jochen Müller</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Gerlingen</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Schillerstraße 18, 70839 Gerlingen, Deutschland</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Schillerstraße 18, 70839 Gerlingen</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>+49 7156 22242</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Sanitärinstallateur</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H13" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
@@ -1014,9 +1008,9 @@
           <t>Ludwigsburg</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
-        <is>
-          <t>Mauserstraße 17, 71640 Ludwigsburg, Deutschland</t>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Mauserstraße 17, 71640 Ludwigsburg</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -1034,53 +1028,53 @@
           <t>4.4 ★</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="n">
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Kurt Knorr GmbH &amp; Co. KG</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Bietigheim-Bissingen</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Bahnhofstraße 105/1, 74321 Bietigheim-Bissingen, Deutschland</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>Bahnhofstraße 105/1, 74321 Bietigheim-Bissingen</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>+49 7142 51191</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="4" t="inlineStr">
         <is>
           <t>Sanitärinstallateur</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>4.9 ★</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -1094,9 +1088,9 @@
           <t>Gerlingen</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Meterstraße 5, 70839 Gerlingen, Deutschland</t>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Meterstraße 5, 70839 Gerlingen</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1114,53 +1108,53 @@
           <t>4.6 ★</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="n">
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>Frank Breuer Installationen</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>Pleidelsheim</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Primelweg 4, 74385 Pleidelsheim, Deutschland</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Primelweg 4, 74385 Pleidelsheim</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
         <is>
           <t>+49 7144 886567</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Sanitärinstallateur</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>4.9 ★</t>
         </is>
       </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
@@ -1174,9 +1168,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>Zweibrücker Str. 15, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Zweibrücker Str. 15, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -1194,53 +1188,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="5" t="n">
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>Verputzarbeiten Knauth e.K.</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Berwartsteinstraße 27, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Berwartsteinstraße 27, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
         <is>
           <t>+49 6341 32393</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>Auftragnehmer</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>4.3 ★</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
@@ -1250,7 +1244,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="2" t="inlineStr">
         <is>
           <t>+49 1515 3406489</t>
@@ -1266,53 +1260,53 @@
           <t>–</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="5" t="n">
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="28" customHeight="1">
+      <c r="A21" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>wahl project GmbH</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>Reutlingen</t>
         </is>
       </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Bayernstraße 18, 72768 Reutlingen, Deutschland</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>Bayernstraße 18, 72768 Reutlingen</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
         <is>
           <t>+49 7121 143090</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Maler</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
@@ -1326,9 +1320,9 @@
           <t>Kirchberg an der Murr</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Danziger Str. 23, 71737 Kirchberg an der Murr, Deutschland</t>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Danziger Str. 23, 71737 Kirchberg an der Murr</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1346,45 +1340,45 @@
           <t>–</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="5" t="n">
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Malermeistebetrieb Jürgen Glass</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr"/>
-      <c r="D23" s="6" t="inlineStr"/>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr"/>
+      <c r="D23" s="4" t="inlineStr"/>
+      <c r="E23" s="4" t="inlineStr">
         <is>
           <t>+49 177 8211470</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>Maler</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="H23" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
@@ -1398,9 +1392,9 @@
           <t>Berg (Pfalz)</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
-        <is>
-          <t>Schubertstraße 4, 76768 Berg (Pfalz), Deutschland</t>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Schubertstraße 4, 76768 Berg (Pfalz)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1418,53 +1412,53 @@
           <t>–</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="5" t="n">
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>Maler Dausch</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>Dahn</t>
         </is>
       </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Bergstraße 1a, 66994 Dahn, Deutschland</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Bergstraße 1a, 66994 Dahn</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
         <is>
           <t>+49 6391 2572</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="4" t="inlineStr">
         <is>
           <t>Maler</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H25" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
@@ -1478,9 +1472,9 @@
           <t>Möglingen</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
-        <is>
-          <t>Eugenstraße 6, 71696 Möglingen, Deutschland</t>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Eugenstraße 6, 71696 Möglingen</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1498,53 +1492,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="5" t="n">
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>Franz-Josef Müller</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>Rastatt</t>
         </is>
       </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Am Altrhein 16, 76437 Rastatt, Deutschland</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Am Altrhein 16, 76437 Rastatt</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>+49 7222 200915</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="4" t="inlineStr">
         <is>
           <t>Sanitärinstallateur</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>4.3 ★</t>
         </is>
       </c>
-      <c r="H27" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
@@ -1558,9 +1552,9 @@
           <t>Rheinstetten</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>Allmendweg 4, 76287 Rheinstetten, Deutschland</t>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Allmendweg 4, 76287 Rheinstetten</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1578,53 +1572,53 @@
           <t>4.5 ★</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="5" t="n">
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="4" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>Dietmar Hermann GmbH</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>Karlsruhe</t>
         </is>
       </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Am Steinhäusle 37, 76228 Karlsruhe, Deutschland</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Am Steinhäusle 37, 76228 Karlsruhe</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>+49 721 45275</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>Sanitärinstallateur</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>3.7 ★</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
@@ -1638,9 +1632,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Queichheimer Hauptstraße 89, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Queichheimer Hauptstraße 89, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -1658,53 +1652,53 @@
           <t>4.7 ★</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="5" t="n">
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="4" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>Volker Braun Klemptnerei Dachdeckerei</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Queichheimer Hauptstraße 182, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>Queichheimer Hauptstraße 182, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
         <is>
           <t>+49 6341 54311</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
@@ -1718,9 +1712,9 @@
           <t>Landau an der Isar</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Gewerbegebiet Straubinger Straße/Lindenstraße, Straubinger Str. 58, 94405 Landau an der Isar, Deutschland</t>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbegebiet Straubinger Straße/Lindenstraße, Straubinger Str. 58, 94405 Landau an der Isar</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1738,53 +1732,53 @@
           <t>4.2 ★</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="5" t="n">
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="A33" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Dachdeckermeister Markus Leber</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>Pfinztal</t>
         </is>
       </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Wesebachstraße 22, 76327 Pfinztal, Deutschland</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Wesebachstraße 22, 76327 Pfinztal</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
         <is>
           <t>+49 7240 7578</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G33" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H33" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
@@ -1798,9 +1792,9 @@
           <t>Bolanden</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Klosterwiesen 9, 67295 Bolanden, Deutschland</t>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Klosterwiesen 9, 67295 Bolanden</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -1818,53 +1812,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="5" t="n">
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1">
+      <c r="A35" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>Dach und Holzbau Saks</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>Hohen-Sülzen</t>
         </is>
       </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>An d. Pfarrwiese 2, 67591 Hohen-Sülzen, Deutschland</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>An d. Pfarrwiese 2, 67591 Hohen-Sülzen</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>+49 176 70468997</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G35" s="4" t="inlineStr">
         <is>
           <t>4.8 ★</t>
         </is>
       </c>
-      <c r="H35" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
@@ -1878,9 +1872,9 @@
           <t>Lampertheim</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>Alte Viernheimer Str. 39, 68623 Lampertheim, Deutschland</t>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Alte Viernheimer Str. 39, 68623 Lampertheim</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -1898,53 +1892,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="5" t="n">
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1">
+      <c r="A37" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>Meisterbau &amp; Dach GmbH</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>Rockenhausen</t>
         </is>
       </c>
-      <c r="D37" s="6" t="inlineStr">
-        <is>
-          <t>Langenwaldstraße 14, 67806 Rockenhausen, Deutschland</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>Langenwaldstraße 14, 67806 Rockenhausen</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
         <is>
           <t>+49 6361 458424</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G37" s="4" t="inlineStr">
         <is>
           <t>4.7 ★</t>
         </is>
       </c>
-      <c r="H37" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="28" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
@@ -1958,9 +1952,9 @@
           <t>Monsheim</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>Hauptstraße 135, 67590 Monsheim, Deutschland</t>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Hauptstraße 135, 67590 Monsheim</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -1978,53 +1972,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="5" t="n">
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="28" customHeight="1">
+      <c r="A39" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Egelhofer Dachdeckerei GmbH</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Falkenstein</t>
         </is>
       </c>
-      <c r="D39" s="6" t="inlineStr">
-        <is>
-          <t>Kreuzweg 2, 67808 Falkenstein, Deutschland</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>Kreuzweg 2, 67808 Falkenstein</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
         <is>
           <t>+49 6302 5414</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F39" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H39" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1">
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="28" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
@@ -2038,9 +2032,9 @@
           <t>Hefersweiler</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Relsberger Str. 1, 67753 Hefersweiler, Deutschland</t>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Relsberger Str. 1, 67753 Hefersweiler</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -2058,53 +2052,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="5" t="n">
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="4" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B41" s="4" t="inlineStr">
         <is>
           <t>MD-Bedachungen &amp; Abdichtungstechnik</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>Kuppenheim</t>
         </is>
       </c>
-      <c r="D41" s="6" t="inlineStr">
-        <is>
-          <t>Bernsteinweg, 76456 Kuppenheim, Deutschland</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>Bernsteinweg, 76456 Kuppenheim</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
         <is>
           <t>+49 176 80768641</t>
         </is>
       </c>
-      <c r="F41" s="5" t="inlineStr">
+      <c r="F41" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G41" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H41" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="18" customHeight="1">
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="28" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
@@ -2118,9 +2112,9 @@
           <t>Durmersheim</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Ob. Bahnhofstraße 12, 76448 Durmersheim, Deutschland</t>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Ob. Bahnhofstraße 12, 76448 Durmersheim</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -2138,53 +2132,53 @@
           <t>3.3 ★</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="5" t="n">
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="28" customHeight="1">
+      <c r="A43" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B43" s="4" t="inlineStr">
         <is>
           <t>Nehr Dach- und Abdichtungstechnik</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>Rheinstetten</t>
         </is>
       </c>
-      <c r="D43" s="6" t="inlineStr">
-        <is>
-          <t>Auer Str. 44, 76287 Rheinstetten, Deutschland</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Auer Str. 44, 76287 Rheinstetten</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
         <is>
           <t>+49 7242 9347485</t>
         </is>
       </c>
-      <c r="F43" s="5" t="inlineStr">
+      <c r="F43" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G43" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H43" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="28" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
@@ -2198,9 +2192,9 @@
           <t>Karlsruhe</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Pfalzstraße 12, 76189 Karlsruhe, Deutschland</t>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Pfalzstraße 12, 76189 Karlsruhe</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -2218,53 +2212,53 @@
           <t>1.8 ★</t>
         </is>
       </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="5" t="n">
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="28" customHeight="1">
+      <c r="A45" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B45" s="4" t="inlineStr">
         <is>
           <t>Rolf Luther</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>Marxzell</t>
         </is>
       </c>
-      <c r="D45" s="6" t="inlineStr">
-        <is>
-          <t>Dekan-Fellhauer-Straße 9, 76359 Marxzell, Deutschland</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Dekan-Fellhauer-Straße 9, 76359 Marxzell</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>+49 7248 1416</t>
         </is>
       </c>
-      <c r="F45" s="5" t="inlineStr">
+      <c r="F45" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G45" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="28" customHeight="1">
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
@@ -2278,9 +2272,9 @@
           <t>Ötigheim</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>Hildastraße 19, 76470 Ötigheim, Deutschland</t>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Hildastraße 19, 76470 Ötigheim</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -2298,53 +2292,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="5" t="n">
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="28" customHeight="1">
+      <c r="A47" s="4" t="n">
         <v>46</v>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
         <is>
           <t>Landesinnungsverband des Dachdeckerhandwerks Baden-Württemberg</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Karlsruhe</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
-        <is>
-          <t>Rüppurrer Str. 13, 76137 Karlsruhe, Deutschland</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Rüppurrer Str. 13, 76137 Karlsruhe</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>+49 721 9338010</t>
         </is>
       </c>
-      <c r="F47" s="5" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>Dachdecker</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="H47" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="28" customHeight="1">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
@@ -2358,9 +2352,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>Nordring 30, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Nordring 30, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
@@ -2378,53 +2372,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="5" t="n">
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="28" customHeight="1">
+      <c r="A49" s="4" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
         <is>
           <t>Klaus Ritzmann KFZ-Reparatur</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Am bhf 16, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Am bhf 16, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>+49 6341 60619</t>
         </is>
       </c>
-      <c r="F49" s="5" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G49" s="4" t="inlineStr">
         <is>
           <t>4.8 ★</t>
         </is>
       </c>
-      <c r="H49" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="18" customHeight="1">
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="28" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
@@ -2438,9 +2432,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>Im Grein 16, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Im Grein 16, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -2458,53 +2452,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="5" t="n">
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="28" customHeight="1">
+      <c r="A51" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="5" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
         <is>
           <t>Schlichting KFZ Reparaturen</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>Im Justus 5, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>Im Justus 5, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>+49 6341 4309</t>
         </is>
       </c>
-      <c r="F51" s="5" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G51" s="5" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>4.7 ★</t>
         </is>
       </c>
-      <c r="H51" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="28" customHeight="1">
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
@@ -2518,9 +2512,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Helmbachstraße 2, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Helmbachstraße 2, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
@@ -2538,53 +2532,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="5" t="n">
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="28" customHeight="1">
+      <c r="A53" s="4" t="n">
         <v>52</v>
       </c>
-      <c r="B53" s="5" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
         <is>
           <t>Neuhart Kfz.-Werkstatt</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Hinterweidenthal</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
-        <is>
-          <t>Industriegebiet 1, 66999 Hinterweidenthal, Deutschland</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Industriegebiet 1, 66999 Hinterweidenthal</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>+49 6396 1711</t>
         </is>
       </c>
-      <c r="F53" s="5" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>4.6 ★</t>
         </is>
       </c>
-      <c r="H53" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="28" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
@@ -2598,9 +2592,9 @@
           <t>Dahn</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Gewerbepark Neudahn 2, 66994 Dahn, Deutschland</t>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Gewerbepark Neudahn 2, 66994 Dahn</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -2618,53 +2612,53 @@
           <t>4.8 ★</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="5" t="n">
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="28" customHeight="1">
+      <c r="A55" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="B55" s="5" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
         <is>
           <t>Hans-Dieter Gein</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D55" s="6" t="inlineStr">
-        <is>
-          <t>Fassendeichstraße 6, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E55" s="5" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Fassendeichstraße 6, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>+49 6341 959926</t>
         </is>
       </c>
-      <c r="F55" s="5" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G55" s="5" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>4.5 ★</t>
         </is>
       </c>
-      <c r="H55" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="18" customHeight="1">
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="28" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
@@ -2678,9 +2672,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Weißenburger Str. 57, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Weißenburger Str. 57, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -2698,53 +2692,53 @@
           <t>4.7 ★</t>
         </is>
       </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="5" t="n">
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="28" customHeight="1">
+      <c r="A57" s="4" t="n">
         <v>56</v>
       </c>
-      <c r="B57" s="5" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
         <is>
           <t>Kfz Werkstatt Merz</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Billigheim-Ingenheim</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Hauptstraße 44, 76831 Billigheim-Ingenheim, Deutschland</t>
-        </is>
-      </c>
-      <c r="E57" s="5" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Hauptstraße 44, 76831 Billigheim-Ingenheim</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="F57" s="5" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>4.7 ★</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="18" customHeight="1">
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="28" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
@@ -2758,9 +2752,9 @@
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>Im Wolfangel 2, 76829 Landau in der Pfalz, Deutschland</t>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Im Wolfangel 2, 76829 Landau in der Pfalz</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -2778,53 +2772,53 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="5" t="n">
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="28" customHeight="1">
+      <c r="A59" s="4" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="5" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>Saab-Zentrum-Südpfalz GmbH</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D59" s="6" t="inlineStr">
-        <is>
-          <t>Lise-Meitner-Straße 2, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Lise-Meitner-Straße 2, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>+49 6341 510999</t>
         </is>
       </c>
-      <c r="F59" s="5" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G59" s="5" t="inlineStr">
+      <c r="G59" s="4" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
-      <c r="H59" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="18" customHeight="1">
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
@@ -2838,9 +2832,9 @@
           <t>Ramberg</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
-        <is>
-          <t>Theo-Klein-Straße 6, 76857 Ramberg, Deutschland</t>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Theo-Klein-Straße 6, 76857 Ramberg</t>
         </is>
       </c>
       <c r="E60" s="2" t="inlineStr">
@@ -2858,53 +2852,53 @@
           <t>4.9 ★</t>
         </is>
       </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="5" t="n">
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1">
+      <c r="A61" s="4" t="n">
         <v>60</v>
       </c>
-      <c r="B61" s="5" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
         <is>
           <t>AIC Ahfir</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Landau in der Pfalz</t>
         </is>
       </c>
-      <c r="D61" s="6" t="inlineStr">
-        <is>
-          <t>Fichtenstraße 7, 76829 Landau in der Pfalz, Deutschland</t>
-        </is>
-      </c>
-      <c r="E61" s="5" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Fichtenstraße 7, 76829 Landau in der Pfalz</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t>+49 6341 51232</t>
         </is>
       </c>
-      <c r="F61" s="5" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t>3 ★</t>
         </is>
       </c>
-      <c r="H61" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="18" customHeight="1">
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1">
       <c r="A62" s="2" t="n">
         <v>61</v>
       </c>
@@ -2918,9 +2912,9 @@
           <t>Frankweiler</t>
         </is>
       </c>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>In d. Plenk 1, 76833 Frankweiler, Deutschland</t>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>In d. Plenk 1, 76833 Frankweiler</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -2938,53 +2932,53 @@
           <t>4.9 ★</t>
         </is>
       </c>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="5" t="n">
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1">
+      <c r="A63" s="4" t="n">
         <v>62</v>
       </c>
-      <c r="B63" s="5" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>KFZ-Werkstatt Liebl</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>Landau an der Isar</t>
         </is>
       </c>
-      <c r="D63" s="6" t="inlineStr">
-        <is>
-          <t>Straubinger Str. 79, 94405 Landau an der Isar, Deutschland</t>
-        </is>
-      </c>
-      <c r="E63" s="5" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Straubinger Str. 79, 94405 Landau an der Isar</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>+49 9951 6821</t>
         </is>
       </c>
-      <c r="F63" s="5" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G63" s="5" t="inlineStr">
+      <c r="G63" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H63" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="18" customHeight="1">
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1">
       <c r="A64" s="2" t="n">
         <v>63</v>
       </c>
@@ -2998,9 +2992,9 @@
           <t>Landau an der Isar</t>
         </is>
       </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Bahnhofstraße 30, 94405 Landau an der Isar, Deutschland</t>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Bahnhofstraße 30, 94405 Landau an der Isar</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -3018,53 +3012,53 @@
           <t>4.8 ★</t>
         </is>
       </c>
-      <c r="H64" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="5" t="n">
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1">
+      <c r="A65" s="4" t="n">
         <v>64</v>
       </c>
-      <c r="B65" s="5" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>Fahrzeugtechnik Papp Michel</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Durmersheim</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Draisstraße 8/2, 76448 Durmersheim, Deutschland</t>
-        </is>
-      </c>
-      <c r="E65" s="5" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Draisstraße 8/2, 76448 Durmersheim</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>+49 7245 9024664</t>
         </is>
       </c>
-      <c r="F65" s="5" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr">
         <is>
           <t>Autowerkstatt</t>
         </is>
       </c>
-      <c r="G65" s="5" t="inlineStr">
+      <c r="G65" s="4" t="inlineStr">
         <is>
           <t>4.8 ★</t>
         </is>
       </c>
-      <c r="H65" s="7" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="18" customHeight="1">
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="28" customHeight="1">
       <c r="A66" s="2" t="n">
         <v>65</v>
       </c>
@@ -3078,9 +3072,9 @@
           <t>Gaggenau</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Wiesentalstraße 1, 76571 Gaggenau, Deutschland</t>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Wiesentalstraße 1, 76571 Gaggenau</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
@@ -3098,47 +3092,47 @@
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H66" s="4" t="inlineStr">
-        <is>
-          <t>Maps öffnen</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="5" t="n">
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>Maps öffnen</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="28" customHeight="1">
+      <c r="A67" s="4" t="n">
         <v>66</v>
       </c>
-      <c r="B67" s="5" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
         <is>
           <t>SEN - (Smart Repair &amp; Spot Repair)</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>Karlsruhe</t>
         </is>
       </c>
-      <c r="D67" s="6" t="inlineStr">
-        <is>
-          <t>Industriestraße 11, 76189 Karlsruhe, Deutschland</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Industriestraße 11, 76189 Karlsruhe</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t>+49 179 3709890</t>
         </is>
       </c>
-      <c r="F67" s="5" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t>Fahrzeuglackiererei</t>
         </is>
       </c>
-      <c r="G67" s="5" t="inlineStr">
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t>5 ★</t>
         </is>
       </c>
-      <c r="H67" s="7" t="inlineStr">
+      <c r="H67" s="5" t="inlineStr">
         <is>
           <t>Maps öffnen</t>
         </is>

</xml_diff>